<commit_message>
Barefoot client schedule: 36-month position nets off the upfront build and connection fee
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_Detailed_Cost_Schedule_2026-09-29.xlsx
+++ b/proposals/Barefoot_Detailed_Cost_Schedule_2026-09-29.xlsx
@@ -553,6 +553,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -725,6 +726,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="5" t="inlineStr">
@@ -844,6 +846,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="5" t="inlineStr">
@@ -980,6 +983,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="n"/>
       <c r="B28" s="5" t="inlineStr">
@@ -1095,6 +1099,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
         <is>
@@ -1128,6 +1133,7 @@
         <v/>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="16" t="inlineStr">
         <is>
@@ -1173,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -1196,6 +1202,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -1293,6 +1300,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
@@ -1372,6 +1380,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
@@ -1412,7 +1421,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Saving over the 36-month agreement</t>
+          <t>Saving on the monthly bill over 36 months</t>
         </is>
       </c>
       <c r="C20" s="23">
@@ -1420,6 +1429,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
@@ -1437,6 +1447,79 @@
         <is>
           <t>Payable once the link is installed</t>
         </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>The 36-month agreement, with the build included</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Saving on the monthly bill over 36 months</t>
+        </is>
+      </c>
+      <c r="C25" s="15">
+        <f>C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Less: network build, paid up front (incl. VAT)</t>
+        </is>
+      </c>
+      <c r="C26" s="15">
+        <f>-'Detailed Cost Schedule'!E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Less: Vodacom once-off connection fee (incl. VAT)</t>
+        </is>
+      </c>
+      <c r="C27" s="15">
+        <f>-C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Net position at the end of the 36 months — build fully paid, network owned</t>
+        </is>
+      </c>
+      <c r="C28" s="21">
+        <f>SUM(C25:C27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Build and connection fee recovered from the saving after (months)</t>
+        </is>
+      </c>
+      <c r="C29" s="24">
+        <f>-(C26+C27)/C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Every year after that, at today's prices</t>
+        </is>
+      </c>
+      <c r="C30" s="15">
+        <f>C17*12</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Barefoot client schedule: labour stated per building at R750/hr (28 buildings x 2 h) plus backbone hours; survey/documentation lines removed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_Detailed_Cost_Schedule_2026-09-29.xlsx
+++ b/proposals/Barefoot_Detailed_Cost_Schedule_2026-09-29.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>25031.83</v>
+        <v>25006.79</v>
       </c>
       <c r="E6" s="9">
         <f>C6*D6</f>
@@ -631,7 +631,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>9637.26</v>
+        <v>9627.58</v>
       </c>
       <c r="E7" s="9">
         <f>C7*D7</f>
@@ -656,7 +656,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>3651.23</v>
+        <v>3647.57</v>
       </c>
       <c r="E8" s="9">
         <f>C8*D8</f>
@@ -677,7 +677,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>9102.49</v>
+        <v>9093.35</v>
       </c>
       <c r="E9" s="9">
         <f>C9*D9</f>
@@ -698,7 +698,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>29527.12</v>
+        <v>29497.48</v>
       </c>
       <c r="E10" s="9">
         <f>C10*D10</f>
@@ -746,7 +746,7 @@
         <v>15</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>3123.29</v>
+        <v>3120.15</v>
       </c>
       <c r="E14" s="9">
         <f>C14*D14</f>
@@ -771,7 +771,7 @@
         <v>10</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>3123.29</v>
+        <v>3120.15</v>
       </c>
       <c r="E15" s="9">
         <f>C15*D15</f>
@@ -796,7 +796,7 @@
         <v>25</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>512.01</v>
+        <v>511.5</v>
       </c>
       <c r="E16" s="9">
         <f>C16*D16</f>
@@ -817,7 +817,7 @@
         <v>1000</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>13.65</v>
+        <v>13.64</v>
       </c>
       <c r="E17" s="9">
         <f>C17*D17</f>
@@ -865,7 +865,7 @@
         <v>22</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>1166.26</v>
+        <v>1165.09</v>
       </c>
       <c r="E21" s="9">
         <f>C21*D21</f>
@@ -890,7 +890,7 @@
         <v>4</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>2144.77</v>
+        <v>2142.62</v>
       </c>
       <c r="E22" s="9">
         <f>C22*D22</f>
@@ -915,7 +915,7 @@
         <v>2</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>2160.7</v>
+        <v>2158.53</v>
       </c>
       <c r="E23" s="9">
         <f>C23*D23</f>
@@ -936,7 +936,7 @@
         <v>2</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>739.58</v>
+        <v>738.83</v>
       </c>
       <c r="E24" s="9">
         <f>C24*D24</f>
@@ -957,7 +957,7 @@
         <v>4</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>682.6900000000001</v>
+        <v>682</v>
       </c>
       <c r="E25" s="9">
         <f>C25*D25</f>
@@ -980,7 +980,7 @@
       <c r="A28" s="4" t="n"/>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Installation, commissioning and handover</t>
+          <t>Installation and commissioning</t>
         </is>
       </c>
       <c r="C28" s="4" t="n"/>
@@ -994,14 +994,14 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Site survey, RF design and link planning</t>
+          <t>Mast, base station, sector antennas, cabinet and solar power system — installation and commissioning (hours)</t>
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>5120.15</v>
+        <v>750</v>
       </c>
       <c r="E29" s="9">
         <f>C29*D29</f>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Completed 22 Sep 2026</t>
+          <t>Two-technician team, at R750 per hour</t>
         </is>
       </c>
     </row>
@@ -1019,14 +1019,14 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Installation — two-technician team: mast, radios, access points, cabling and power (25 buildings)</t>
+          <t>Per building: subscriber radio mounted on the building, cable pulled in, Wi-Fi access point mounted on the ceiling and tested (28 buildings × 2 hours)</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>10240.3</v>
+        <v>750</v>
       </c>
       <c r="E30" s="9">
         <f>C30*D30</f>
@@ -1034,130 +1034,88 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Per day</t>
+          <t>At R750 per hour</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Commissioning, link testing and Wi-Fi coverage verification</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="9" t="n">
-        <v>5120.15</v>
-      </c>
-      <c r="E31" s="9">
-        <f>C31*D31</f>
-        <v/>
-      </c>
-      <c r="F31" s="10" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Documentation, training and handover</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="9" t="n">
-        <v>2563.81</v>
-      </c>
-      <c r="E32" s="9">
-        <f>C32*D32</f>
-        <v/>
-      </c>
-      <c r="F32" s="10" t="inlineStr"/>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal — Installation and commissioning</t>
+        </is>
+      </c>
+      <c r="E31" s="12">
+        <f>SUM(E29:E30)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal — Installation, commissioning and handover</t>
-        </is>
-      </c>
-      <c r="E33" s="12">
-        <f>SUM(E29:E32)</f>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL — network build, excluding VAT</t>
+        </is>
+      </c>
+      <c r="E33" s="14">
+        <f>E11+E18+E26+E31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>VAT at 15%</t>
+        </is>
+      </c>
+      <c r="E34" s="15">
+        <f>E33*0.15</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>TOTAL — network build, excluding VAT</t>
+          <t>TOTAL — network build, including VAT</t>
         </is>
       </c>
       <c r="E35" s="14">
-        <f>E11+E18+E26+E33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>VAT at 15%</t>
-        </is>
-      </c>
-      <c r="E36" s="15">
-        <f>E35*0.15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>TOTAL — network build, including VAT</t>
-        </is>
-      </c>
-      <c r="E37" s="14">
-        <f>E35+E36</f>
-        <v/>
+        <f>E33+E34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>Payment terms: 50% on order (secures the equipment allocation and places the order), 50% on commissioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Ownership: all equipment, the mast, the cabinet and the power system are the property of Barefoot Addo Elephant Lodge (Pty) Ltd on handover.</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>Payment terms: 50% on order (secures the equipment allocation and places the order), 50% on commissioning.</t>
+          <t>Included: delivery to site, installation, configuration and testing of every item above. Manufacturer warranties apply (Cambium 12 months; extended 2-year cover available as an option on request).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>Ownership: all equipment, the mast, the cabinet and the power system are the property of Barefoot Addo Elephant Lodge (Pty) Ltd on handover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>Included: design, delivery to site, installation, configuration, testing, documentation and training. Manufacturer warranties apply (Cambium 12 months; extended 2-year cover available as an option on request).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="B42" s="16" t="inlineStr">
-        <is>
           <t>Not included: the Vodacom carrier link (see Monthly Costs), trenching or civil works beyond the mast plinth, Eskom connections, and any building works.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B37:F37"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B39:F39"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B38:F38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1444,7 +1402,7 @@
         </is>
       </c>
       <c r="C24" s="15">
-        <f>-'Detailed Cost Schedule'!E37</f>
+        <f>-'Detailed Cost Schedule'!E35</f>
         <v/>
       </c>
     </row>
@@ -1539,7 +1497,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>'Detailed Cost Schedule'!E37</f>
+        <f>'Detailed Cost Schedule'!E35</f>
         <v/>
       </c>
     </row>

</xml_diff>